<commit_message>
add: create test file no.13
</commit_message>
<xml_diff>
--- a/docs/ScenarioTest.xlsx
+++ b/docs/ScenarioTest.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ltmb20260008/work/dog/generate_dummy_data/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{232B81B8-CD7A-2247-888C-6B91F3AFD23E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{156A5DB2-2B9D-B244-9045-F665577064E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{15BD4E46-EBEB-47CA-9D81-183BAD66E7E6}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="481">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="587" uniqueCount="480">
   <si>
     <t>作成日</t>
   </si>
@@ -196,9 +196,6 @@
     <t>正常日次 8 ファイル取込</t>
   </si>
   <si>
-    <t>対象日の 8 ファイルを取込先 tmp_* へ正常ロードできる</t>
-  </si>
-  <si>
     <t>データA：A-01
 データB：B-01
 データC：C-01</t>
@@ -252,9 +249,6 @@
   </si>
   <si>
     <t>同一日付・同一データの再実行でも二重反映しない</t>
-  </si>
-  <si>
-    <t>No.4の同じファイルで可</t>
   </si>
   <si>
     <t>1.同一対象日データを一度正常取込済みであること
@@ -419,50 +413,18 @@
     <t>異常データ制御</t>
   </si>
   <si>
-    <t>型変換エラー継続</t>
-  </si>
-  <si>
-    <t>変換不能な日付・数値が来ても該当項目を NULL として処理継続できる</t>
-  </si>
-  <si>
     <t>データA：A-11
 データC：C-08</t>
   </si>
   <si>
-    <t>1.型変換不能値を含む状態で process_trn_approval_mobile を実行する
-2.完了後に変換エラーログを確認する
-3.App DB の trn_approval_mobile で該当項目の値を確認する</t>
-  </si>
-  <si>
-    <t>1.パイプライン全体が継続または想定どおり完了していること
-2.変換不能な日付・数値のエラーがログに記録されていること
-3.該当項目は NULL で反映され、trn_approval_mobile は 期待値（C）どおりであること</t>
-  </si>
-  <si>
     <t>14</t>
   </si>
   <si>
     <t>2-2-2</t>
-  </si>
-  <si>
-    <t>重複キー継続</t>
-  </si>
-  <si>
-    <t>同一キー重複時に新しいデータを正として継続できる</t>
   </si>
   <si>
     <t>データA：A-12
 データC：C-09</t>
-  </si>
-  <si>
-    <t>1.重複キーを含む状態で process_trn_approval_mobile を実行する
-2.完了後に App DB の trn_approval_mobile を確認する
-3.同一 approval_id の件数と採用された値を確認する</t>
-  </si>
-  <si>
-    <t>1.パイプラインが異常終了せず処理継続していること
-2.同一 approval_id が二重登録されていないこと
-3.優先条件上の新しいデータが App DB の期待値（C）として採用されていること</t>
   </si>
   <si>
     <t>15</t>
@@ -1475,17 +1437,6 @@
 ・各 process の処理時間を記録するモニタリング環境が整備されていること</t>
   </si>
   <si>
-    <t>1.Kiwi に yyyyMMdd の日次 8 ファイル一式が配置済みであること
-※ ファイル名の日付はテスト日に変更して行うこと</t>
-    <rPh sb="50" eb="52">
-      <t xml:space="preserve">ヒヅケ </t>
-    </rPh>
-    <rPh sb="58" eb="60">
-      <t xml:space="preserve">ヘンコウ </t>
-    </rPh>
-    <phoneticPr fontId="2"/>
-  </si>
-  <si>
     <t>1.ADF の extract_daily パイプラインを手動実行する
 2.8 ファイル分の activity が完了していることを確認する
 3.ETL DB の tmp_* または tmp_diff_* の件数と代表キーを確認する</t>
@@ -1707,30 +1658,6 @@
   </si>
   <si>
     <t>入力
-A.dwh_test_13_input_YYYYMMDD_DLV_OAI_COM_EIG_KESSAI.csv.gz
-B.dwh_test_13_input_trn_approval_mobile.csv
-期待値
-C.dwh_test_13_output_trn_approval_mobile.csv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1.ETL DB の YYYYMMDD_DLV_OAI_COM_EIG_KESSAI に不正日付・不正数値を含むデータ（A）が入っていること
-2.App DB の trn_approval_mobile に事前データ（B）が登録されていること
-</t>
-  </si>
-  <si>
-    <t>入力
-A.dwh_test_14_input_YYYYMMDD_DLV_OAI_COM_EIG_KESSAI.csv.gz
-B.dwh_test_14_input_trn_approval_mobile.csv
-期待値
-C.dwh_test_14_output_trn_approval_mobile.csv</t>
-  </si>
-  <si>
-    <t>1.ETL DB の YYYYMMDD_DLV_OAI_COM_EIG_KESSAI に同一 決裁番号(approval_id) を持つ 2 行（A）が入っていること
-2.App DB の trn_approval_mobile に事前データ（B）が登録されていること
-3.新旧判定に使う更新日時または優先条件を確認できること</t>
-  </si>
-  <si>
-    <t>入力
 A.dwh_test_07_input_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
 B.dwh_test_07_input_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
 C.dwh_test_07_input_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
@@ -1746,20 +1673,6 @@
 C.dwh_test_24_input_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.csv.gz
 入力: 全量データ
 D.dwh_test_24_input_YYYYMMDD_DLV_OAI_MRS_ITEM.csv.gz</t>
-  </si>
-  <si>
-    <t>1.パイプラインが正常終了していること
-2.空ファイル対象の Copy activity がエラーにならないこと
-3.以下の対象 テーブルは 0 件であること
-・tmp_diff_bfs_entry_informations 
-・tmp_diff_bfs_service_summary_devices
-・tmp_diff_bfs_service_summary_accessories
-・YYYYMMDD_DLV_OAI_SMT_DV_SMT_MST_UNIQ_CORP_IE
-・YYYYMMDD_DLV_OAI_COM_EIG_KESSAI
-・tmp_mars_agency
-・YYYYMMDD_DLV_OAI_MRS_ITEM
-・YYYYMMDD_DLV_OAI_MRS_CMPGN
-　上記テーブルも全て 0 件であること</t>
   </si>
   <si>
     <t>入力
@@ -1782,34 +1695,6 @@
 dwh_test_03_input_YYYYMMDD_DLV_OAI_CST_ORDCSTM.csv.gz
 dwh_test_03_input_YYYYMMDD_DLV_OAI_MRS_ITEM.csv.gz
 dwh_test_03_input_YYYYMMDD_DLV_OAI_MRS_CMPGN.csv.gz</t>
-  </si>
-  <si>
-    <t>入力
-dwh_test_04_input_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_SMT_DV_SMT_MST_UNIQ_CORP_IE.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_COM_EIG_KESSAI.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_CST_ORDCSTM.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_MRS_ITEM.csv.gz
-dwh_test_04_input_YYYYMMDD_DLV_OAI_MRS_CMPGN.csv.gz</t>
-  </si>
-  <si>
-    <t>1.パイプラインが正常終了していること
-2.下記テーブルに対象日データがロードされていること
-tmp_diff_bfs_entry_informations
-tmp_diff_bfs_service_summary_devices
-tmp_diff_bfs_service_summary_accessories
-YYYYMMDD_DLV_OAI_SMT_DV_SMT_MST_UNIQ_CORP_IE
-YYYYMMDD_DLV_OAI_COM_EIG_KESSAI
-tmp_diff_mars_agency
-YYYYMMDD_DLV_OAI_MRS_ITEM
-YYYYMMDD_DLV_OAI_MRS_CMPGN
-3.company_id=TK2458 / approval_id=LS2968483 / entry_number=ENT-20260427-0001 の横断整合を確認できること</t>
-    <rPh sb="22" eb="24">
-      <t xml:space="preserve">カキ </t>
-    </rPh>
-    <phoneticPr fontId="2"/>
   </si>
   <si>
     <t>入力
@@ -2098,6 +1983,133 @@
     <rPh sb="147" eb="148">
       <t xml:space="preserve">フクム </t>
     </rPh>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>型変換エラー失敗</t>
+    <rPh sb="6" eb="8">
+      <t xml:space="preserve">シッパイ </t>
+    </rPh>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>変換不能な日付・数値が来たら失敗で終わる</t>
+    <rPh sb="14" eb="16">
+      <t xml:space="preserve">シッパイ </t>
+    </rPh>
+    <rPh sb="17" eb="18">
+      <t xml:space="preserve">オワル </t>
+    </rPh>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>1.データ(A) にある一部のデータは plannedstartdate の値が日付として正しくない値であること（例、DUMMYDATE, HOGE など）</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t xml:space="preserve">1.データ(A) を設置して、extract_daily を実行し、tmp_diffテーブルに反映する
+2.ADF の process_trn_approval_mobile パイプラインを実行する
+</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>1.パイプラインが異常終了していること
+2.エラー内容から変換失敗のエラーであることが判断できること</t>
+    <rPh sb="25" eb="27">
+      <t>イジョウ _x0000__x0019__x0002__x0007__x0019__x0002__x000E__x001D__x0002__x0013__x001F__x0002__x0018_+_x0002__x0000__x0000__x0000__x0000_</t>
+    </rPh>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>2.データ(A) には 同一の決裁番号(approval_id) を持つ行が入っていること（新旧判定に使う更新日時または優先条件を確認できること）</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>1.パイプラインが異常終了せず処理継続していること
+2.同一 approval_id が二重登録されていないこと</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t xml:space="preserve">A.dwh_test_13_input_YYYYMMDD_DLV_OAI_COM_EIG_KESSAI.csv.gz 
+</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>A.dwh_test_14_input_YYYYMMDD_DLV_OAI_COM_EIG_KESSAI.csv.gz 
+B.dwh_test_14_expect_trn_approval_mobile.csv</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>重複キー継続</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>同一キー重複時に新しいデータを正として継続できる</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>入力
+dwh_test_04_input_YYYYMMDD_DLV_OAI_BFS_BFS_ENTRY_INFO.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_BFS_BFS_SERVICE_SUMMARY4.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_BFS_BFS_ATTACHMENT_SUMMALLY.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_SMT_DV_SMT_MST_UNIQ_CORP_IE.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_COM_EIG_KESSAI.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_CST_ORDCSTM.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_MRS_ITEM.csv.gz
+dwh_test_04_input_YYYYMMDD_DLV_OAI_MRS_CMPGN.csv.gz</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t>対象日の 8 ファイルを取込先 tmp_* へ正常ロードできる</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Kiwi に yyyyMMdd の日次 8 ファイル一式が配置済みであること
+※ ファイル名の日付はテスト日に変更して行うこと
+2.company_id=TK2458 / approval_id=LS2968483 / entry_number=ENT-20260427-0001 の横断整合を確認できること
+</t>
+    <rPh sb="50" eb="52">
+      <t xml:space="preserve">ヒヅケ </t>
+    </rPh>
+    <rPh sb="58" eb="60">
+      <t xml:space="preserve">ヘンコウ </t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>1.パイプラインが正常終了していること
+2.空ファイル対象の Copy activity がエラーにならないこと
+3.以下の対象 テーブルは 0 件であること
+・tmp_diff_bfs_entry_informations 
+・tmp_diff_bfs_service_summary_devices
+・tmp_diff_bfs_service_summary_accessories
+・tmp_diff_corp_customer_info
+・tmp_diff_compass_sales_approval
+・tmp_mars_agency
+・tmp_mars_product
+・tmp_mars_campaign
+　上記テーブルも全て 0 件であること</t>
+    <phoneticPr fontId="13"/>
+  </si>
+  <si>
+    <t xml:space="preserve">1.パイプラインが正常終了していること
+2.下記テーブルに対象日データがロードされていること
+tmp_diff_bfs_entry_informations
+tmp_diff_bfs_service_summary_devices
+tmp_diff_bfs_service_summary_accessories
+tmp_diff_corp_customer_info
+tmp_diff_compass_sales_approval
+tmp_diff_mars_agency
+tmp_mars_product
+tmp_mars_campaign
+</t>
+    <rPh sb="22" eb="24">
+      <t xml:space="preserve">カキ </t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>No.4と同じファイルで可</t>
     <phoneticPr fontId="13"/>
   </si>
 </sst>
@@ -2612,6 +2624,9 @@
     <xf numFmtId="0" fontId="17" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -2626,9 +2641,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2952,30 +2964,30 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="14.25" customHeight="1">
-      <c r="A1" s="47" t="s">
-        <v>415</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
+      <c r="A1" s="48" t="s">
+        <v>404</v>
+      </c>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
     </row>
     <row r="2" spans="1:13">
-      <c r="A2" s="48"/>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
+      <c r="A2" s="49"/>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
     </row>
     <row r="3" spans="1:13">
-      <c r="A3" s="48"/>
-      <c r="B3" s="48"/>
-      <c r="C3" s="48"/>
-      <c r="D3" s="48"/>
-      <c r="E3" s="48"/>
-      <c r="F3" s="48"/>
+      <c r="A3" s="49"/>
+      <c r="B3" s="49"/>
+      <c r="C3" s="49"/>
+      <c r="D3" s="49"/>
+      <c r="E3" s="49"/>
+      <c r="F3" s="49"/>
       <c r="J3" s="32" t="s">
         <v>0</v>
       </c>
@@ -2987,12 +2999,12 @@
       </c>
     </row>
     <row r="4" spans="1:13" ht="49.5" customHeight="1">
-      <c r="A4" s="48"/>
-      <c r="B4" s="48"/>
-      <c r="C4" s="48"/>
-      <c r="D4" s="48"/>
-      <c r="E4" s="48"/>
-      <c r="F4" s="48"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="49"/>
+      <c r="C4" s="49"/>
+      <c r="D4" s="49"/>
+      <c r="E4" s="49"/>
+      <c r="F4" s="49"/>
       <c r="J4" s="33">
         <v>46153</v>
       </c>
@@ -3023,7 +3035,7 @@
         <v>10</v>
       </c>
       <c r="H6" s="4" t="s">
-        <v>431</v>
+        <v>420</v>
       </c>
       <c r="I6" s="4" t="s">
         <v>11</v>
@@ -3061,10 +3073,10 @@
         <v>21</v>
       </c>
       <c r="G7" s="8" t="s">
-        <v>432</v>
+        <v>421</v>
       </c>
       <c r="H7" s="8" t="s">
-        <v>449</v>
+        <v>431</v>
       </c>
       <c r="I7" s="35" t="s">
         <v>22</v>
@@ -3075,8 +3087,8 @@
       <c r="K7" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="36" t="s">
-        <v>440</v>
+      <c r="L7" s="35" t="s">
+        <v>477</v>
       </c>
       <c r="M7" s="8"/>
     </row>
@@ -3099,10 +3111,10 @@
         <v>28</v>
       </c>
       <c r="H8" s="8" t="s">
-        <v>441</v>
+        <v>425</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>433</v>
+        <v>422</v>
       </c>
       <c r="J8" s="8" t="s">
         <v>29</v>
@@ -3134,7 +3146,7 @@
         <v>35</v>
       </c>
       <c r="H9" s="8" t="s">
-        <v>442</v>
+        <v>426</v>
       </c>
       <c r="I9" s="8" t="s">
         <v>36</v>
@@ -3168,744 +3180,744 @@
         <v>21</v>
       </c>
       <c r="G10" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>474</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>476</v>
+      </c>
+      <c r="J10" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>443</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>408</v>
-      </c>
-      <c r="J10" s="8" t="s">
-        <v>45</v>
-      </c>
       <c r="K10" s="8" t="s">
-        <v>409</v>
-      </c>
-      <c r="L10" s="8" t="s">
-        <v>444</v>
+        <v>398</v>
+      </c>
+      <c r="L10" s="35" t="s">
+        <v>478</v>
       </c>
       <c r="M10" s="8"/>
     </row>
     <row r="11" spans="1:13" ht="165" customHeight="1">
       <c r="A11" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>46</v>
-      </c>
-      <c r="B11" s="14" t="s">
-        <v>47</v>
       </c>
       <c r="C11" s="16"/>
       <c r="D11" s="16"/>
       <c r="E11" s="18" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="F11" s="8" t="s">
+      <c r="G11" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="8" t="s">
+      <c r="H11" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="I11" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="H11" s="8" t="s">
-        <v>445</v>
-      </c>
-      <c r="I11" s="8" t="s">
+      <c r="J11" s="8" t="s">
         <v>51</v>
       </c>
-      <c r="J11" s="8" t="s">
+      <c r="K11" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="K11" s="8" t="s">
+      <c r="L11" s="35" t="s">
         <v>53</v>
-      </c>
-      <c r="L11" s="35" t="s">
-        <v>54</v>
       </c>
       <c r="M11" s="8"/>
     </row>
     <row r="12" spans="1:13" ht="195" customHeight="1">
       <c r="A12" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="14" t="s">
         <v>55</v>
-      </c>
-      <c r="B12" s="14" t="s">
-        <v>56</v>
       </c>
       <c r="C12" s="17"/>
       <c r="D12" s="17"/>
       <c r="E12" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="F12" s="8" t="s">
+      <c r="G12" s="8" t="s">
         <v>58</v>
       </c>
-      <c r="G12" s="8" t="s">
+      <c r="H12" s="8" t="s">
+        <v>479</v>
+      </c>
+      <c r="I12" s="35" t="s">
         <v>59</v>
       </c>
-      <c r="H12" s="8" t="s">
+      <c r="J12" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="K12" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="I12" s="35" t="s">
+      <c r="L12" s="8" t="s">
         <v>61</v>
-      </c>
-      <c r="J12" s="8" t="s">
-        <v>416</v>
-      </c>
-      <c r="K12" s="8" t="s">
-        <v>62</v>
-      </c>
-      <c r="L12" s="8" t="s">
-        <v>63</v>
       </c>
       <c r="M12" s="8"/>
     </row>
     <row r="13" spans="1:13" ht="152.25" customHeight="1">
       <c r="A13" s="26" t="s">
+        <v>62</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="15" t="s">
         <v>64</v>
       </c>
-      <c r="B13" s="14" t="s">
+      <c r="D13" s="15" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="E13" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="F13" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="E13" s="18" t="s">
+      <c r="G13" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="H13" s="8" t="s">
+        <v>423</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="J13" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="G13" s="8" t="s">
-        <v>70</v>
-      </c>
-      <c r="H13" s="8" t="s">
-        <v>438</v>
-      </c>
-      <c r="I13" s="8" t="s">
-        <v>428</v>
-      </c>
-      <c r="J13" s="8" t="s">
-        <v>71</v>
-      </c>
       <c r="K13" s="8" t="s">
-        <v>429</v>
+        <v>418</v>
       </c>
       <c r="L13" s="8" t="s">
-        <v>430</v>
+        <v>419</v>
       </c>
       <c r="M13" s="8"/>
     </row>
     <row r="14" spans="1:13" ht="108" customHeight="1">
       <c r="A14" s="26" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C14" s="16"/>
       <c r="D14" s="16"/>
       <c r="E14" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="F14" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="G14" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="F14" s="8" t="s">
+      <c r="H14" s="8" t="s">
+        <v>433</v>
+      </c>
+      <c r="I14" s="35" t="s">
+        <v>462</v>
+      </c>
+      <c r="J14" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="G14" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="H14" s="8" t="s">
-        <v>451</v>
-      </c>
-      <c r="I14" s="35" t="s">
-        <v>480</v>
-      </c>
-      <c r="J14" s="8" t="s">
-        <v>77</v>
-      </c>
       <c r="K14" s="8" t="s">
-        <v>450</v>
+        <v>432</v>
       </c>
       <c r="L14" s="35" t="s">
-        <v>453</v>
+        <v>435</v>
       </c>
       <c r="M14" s="8"/>
     </row>
     <row r="15" spans="1:13" ht="106" customHeight="1">
       <c r="A15" s="26" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C15" s="16"/>
       <c r="D15" s="16"/>
       <c r="E15" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="G15" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="F15" s="8" t="s">
+      <c r="H15" s="8" t="s">
+        <v>434</v>
+      </c>
+      <c r="I15" s="47" t="s">
+        <v>454</v>
+      </c>
+      <c r="J15" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="G15" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="H15" s="8" t="s">
-        <v>452</v>
-      </c>
-      <c r="I15" s="54" t="s">
-        <v>472</v>
-      </c>
-      <c r="J15" s="8" t="s">
-        <v>83</v>
-      </c>
       <c r="K15" s="35" t="s">
-        <v>471</v>
+        <v>453</v>
       </c>
       <c r="L15" s="8" t="s">
-        <v>454</v>
+        <v>436</v>
       </c>
       <c r="M15" s="8"/>
     </row>
     <row r="16" spans="1:13" ht="126" customHeight="1">
       <c r="A16" s="26" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B16" s="14" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C16" s="16"/>
       <c r="D16" s="16"/>
       <c r="E16" s="18" t="s">
+        <v>84</v>
+      </c>
+      <c r="F16" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="G16" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="F16" s="8" t="s">
+      <c r="H16" s="8" t="s">
+        <v>461</v>
+      </c>
+      <c r="I16" s="35" t="s">
+        <v>458</v>
+      </c>
+      <c r="J16" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="G16" s="8" t="s">
-        <v>88</v>
-      </c>
-      <c r="H16" s="8" t="s">
-        <v>479</v>
-      </c>
-      <c r="I16" s="35" t="s">
-        <v>476</v>
-      </c>
-      <c r="J16" s="8" t="s">
-        <v>89</v>
-      </c>
       <c r="K16" s="35" t="s">
-        <v>477</v>
+        <v>459</v>
       </c>
       <c r="L16" s="8" t="s">
-        <v>478</v>
+        <v>460</v>
       </c>
       <c r="M16" s="8"/>
     </row>
     <row r="17" spans="1:13" ht="177" customHeight="1">
       <c r="A17" s="26" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C17" s="16"/>
       <c r="D17" s="16"/>
       <c r="E17" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="F17" s="8" t="s">
+        <v>91</v>
+      </c>
+      <c r="G17" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="F17" s="8" t="s">
+      <c r="H17" s="35" t="s">
+        <v>447</v>
+      </c>
+      <c r="I17" s="35" t="s">
+        <v>454</v>
+      </c>
+      <c r="J17" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="G17" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="H17" s="35" t="s">
-        <v>465</v>
-      </c>
-      <c r="I17" s="35" t="s">
-        <v>472</v>
-      </c>
-      <c r="J17" s="8" t="s">
-        <v>95</v>
-      </c>
       <c r="K17" s="36" t="s">
-        <v>466</v>
+        <v>448</v>
       </c>
       <c r="L17" s="35" t="s">
-        <v>467</v>
+        <v>449</v>
       </c>
       <c r="M17" s="8"/>
     </row>
     <row r="18" spans="1:13" ht="120" customHeight="1">
       <c r="A18" s="26" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C18" s="16"/>
       <c r="D18" s="17"/>
       <c r="E18" s="18" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>440</v>
+      </c>
+      <c r="H18" s="35" t="s">
+        <v>437</v>
+      </c>
+      <c r="I18" s="36" t="s">
+        <v>455</v>
+      </c>
+      <c r="J18" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="F18" s="8" t="s">
-        <v>99</v>
-      </c>
-      <c r="G18" s="8" t="s">
-        <v>458</v>
-      </c>
-      <c r="H18" s="35" t="s">
-        <v>455</v>
-      </c>
-      <c r="I18" s="36" t="s">
-        <v>473</v>
-      </c>
-      <c r="J18" s="8" t="s">
-        <v>100</v>
-      </c>
       <c r="K18" s="36" t="s">
-        <v>457</v>
+        <v>439</v>
       </c>
       <c r="L18" s="36" t="s">
-        <v>456</v>
+        <v>438</v>
       </c>
       <c r="M18" s="8"/>
     </row>
     <row r="19" spans="1:13" ht="121" customHeight="1">
       <c r="A19" s="26" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C19" s="16"/>
       <c r="D19" s="15" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E19" s="18" t="s">
-        <v>104</v>
+        <v>463</v>
       </c>
       <c r="F19" s="8" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
       <c r="G19" s="8" t="s">
-        <v>105</v>
+        <v>464</v>
       </c>
       <c r="H19" s="8" t="s">
-        <v>434</v>
+        <v>470</v>
       </c>
       <c r="I19" s="8" t="s">
-        <v>435</v>
+        <v>465</v>
       </c>
       <c r="J19" s="8" t="s">
-        <v>106</v>
-      </c>
-      <c r="K19" s="8" t="s">
-        <v>107</v>
-      </c>
-      <c r="L19" s="8" t="s">
-        <v>108</v>
+        <v>102</v>
+      </c>
+      <c r="K19" s="36" t="s">
+        <v>466</v>
+      </c>
+      <c r="L19" s="35" t="s">
+        <v>467</v>
       </c>
       <c r="M19" s="8"/>
     </row>
     <row r="20" spans="1:13" ht="134.25" customHeight="1">
       <c r="A20" s="26" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C20" s="17"/>
       <c r="D20" s="17"/>
       <c r="E20" s="18" t="s">
-        <v>111</v>
+        <v>472</v>
       </c>
       <c r="F20" s="8" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G20" s="8" t="s">
-        <v>112</v>
+        <v>473</v>
       </c>
       <c r="H20" s="8" t="s">
-        <v>436</v>
+        <v>471</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>437</v>
+        <v>468</v>
       </c>
       <c r="J20" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="K20" s="8" t="s">
-        <v>114</v>
+        <v>105</v>
+      </c>
+      <c r="K20" s="36" t="s">
+        <v>466</v>
       </c>
       <c r="L20" s="8" t="s">
-        <v>115</v>
+        <v>469</v>
       </c>
       <c r="M20" s="8"/>
     </row>
     <row r="21" spans="1:13" ht="108" customHeight="1">
       <c r="A21" s="26" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="E21" s="18" t="s">
-        <v>469</v>
+        <v>451</v>
       </c>
       <c r="F21" s="8" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="G21" s="8" t="s">
-        <v>468</v>
+        <v>450</v>
       </c>
       <c r="H21" s="8" t="s">
-        <v>463</v>
+        <v>445</v>
       </c>
       <c r="I21" s="8" t="s">
-        <v>474</v>
+        <v>456</v>
       </c>
       <c r="J21" s="8" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="K21" s="8" t="s">
-        <v>462</v>
+        <v>444</v>
       </c>
       <c r="L21" s="8" t="s">
-        <v>461</v>
+        <v>443</v>
       </c>
       <c r="M21" s="8"/>
     </row>
     <row r="22" spans="1:13" ht="121" customHeight="1">
       <c r="A22" s="26" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C22" s="16"/>
       <c r="D22" s="17"/>
       <c r="E22" s="18" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="F22" s="8" t="s">
-        <v>126</v>
+        <v>116</v>
       </c>
       <c r="G22" s="8" t="s">
-        <v>127</v>
+        <v>117</v>
       </c>
       <c r="H22" s="8" t="s">
-        <v>464</v>
+        <v>446</v>
       </c>
       <c r="I22" s="8" t="s">
-        <v>475</v>
+        <v>457</v>
       </c>
       <c r="J22" s="8" t="s">
-        <v>128</v>
+        <v>118</v>
       </c>
       <c r="K22" s="8" t="s">
-        <v>459</v>
+        <v>441</v>
       </c>
       <c r="L22" s="8" t="s">
-        <v>460</v>
+        <v>442</v>
       </c>
       <c r="M22" s="8"/>
     </row>
     <row r="23" spans="1:13" ht="137.25" customHeight="1">
       <c r="A23" s="26" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="D23" s="19" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="E23" s="18" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="F23" s="8" t="s">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="G23" s="8" t="s">
-        <v>470</v>
+        <v>452</v>
       </c>
       <c r="H23" s="8" t="s">
-        <v>446</v>
+        <v>428</v>
       </c>
       <c r="I23" s="8" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="J23" s="8" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="K23" s="35" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
       <c r="L23" s="35" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
       <c r="M23" s="8"/>
     </row>
     <row r="24" spans="1:13" ht="194.25" customHeight="1">
       <c r="A24" s="26" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C24" s="37"/>
       <c r="D24" s="15" t="s">
-        <v>141</v>
+        <v>131</v>
       </c>
       <c r="E24" s="18" t="s">
-        <v>142</v>
+        <v>132</v>
       </c>
       <c r="F24" s="8" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="G24" s="8" t="s">
-        <v>144</v>
+        <v>134</v>
       </c>
       <c r="H24" s="8" t="s">
-        <v>447</v>
+        <v>429</v>
       </c>
       <c r="I24" s="8" t="s">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="J24" s="8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="K24" s="35" t="s">
-        <v>146</v>
+        <v>136</v>
       </c>
       <c r="L24" s="8" t="s">
-        <v>147</v>
+        <v>137</v>
       </c>
       <c r="M24" s="8"/>
     </row>
     <row r="25" spans="1:13" ht="160" customHeight="1">
       <c r="A25" s="26" t="s">
-        <v>148</v>
+        <v>138</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C25" s="16"/>
       <c r="D25" s="16"/>
       <c r="E25" s="18" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="F25" s="8" t="s">
-        <v>151</v>
+        <v>141</v>
       </c>
       <c r="G25" s="8" t="s">
-        <v>152</v>
+        <v>142</v>
       </c>
       <c r="H25" s="8" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="I25" s="8" t="s">
-        <v>154</v>
+        <v>144</v>
       </c>
       <c r="J25" s="8" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="K25" s="8" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="L25" s="38" t="s">
-        <v>418</v>
+        <v>407</v>
       </c>
       <c r="M25" s="8"/>
     </row>
     <row r="26" spans="1:13" ht="139" customHeight="1">
       <c r="A26" s="26" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
       <c r="E26" s="18" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="F26" s="8" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="G26" s="8" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="H26" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I26" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="J26" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="I26" s="8" t="s">
-        <v>162</v>
-      </c>
-      <c r="J26" s="8" t="s">
-        <v>163</v>
-      </c>
       <c r="K26" s="8" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="L26" s="8" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="M26" s="8"/>
     </row>
     <row r="27" spans="1:13" ht="110.25" customHeight="1">
       <c r="A27" s="26" t="s">
-        <v>166</v>
+        <v>156</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="C27" s="16"/>
       <c r="D27" s="17"/>
       <c r="E27" s="18" t="s">
-        <v>168</v>
+        <v>158</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>169</v>
+        <v>159</v>
       </c>
       <c r="G27" s="8" t="s">
-        <v>170</v>
+        <v>160</v>
       </c>
       <c r="H27" s="8" t="s">
+        <v>143</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>401</v>
+      </c>
+      <c r="J27" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="I27" s="8" t="s">
-        <v>412</v>
-      </c>
-      <c r="J27" s="8" t="s">
-        <v>163</v>
-      </c>
       <c r="K27" s="8" t="s">
-        <v>171</v>
+        <v>161</v>
       </c>
       <c r="L27" s="8" t="s">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="M27" s="8"/>
     </row>
     <row r="28" spans="1:13" ht="87" customHeight="1">
       <c r="A28" s="26" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C28" s="16"/>
       <c r="D28" s="19" t="s">
-        <v>175</v>
+        <v>165</v>
       </c>
       <c r="E28" s="18" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>177</v>
+        <v>167</v>
       </c>
       <c r="G28" s="8" t="s">
-        <v>178</v>
+        <v>168</v>
       </c>
       <c r="H28" s="8" t="s">
-        <v>153</v>
+        <v>143</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>179</v>
+        <v>169</v>
       </c>
       <c r="J28" s="8" t="s">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="K28" s="8" t="s">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="L28" s="8" t="s">
-        <v>182</v>
+        <v>172</v>
       </c>
       <c r="M28" s="8"/>
     </row>
     <row r="29" spans="1:13" ht="162" customHeight="1">
       <c r="A29" s="26" t="s">
-        <v>183</v>
+        <v>173</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C29" s="16"/>
       <c r="D29" s="15" t="s">
-        <v>185</v>
+        <v>175</v>
       </c>
       <c r="E29" s="18" t="s">
-        <v>186</v>
+        <v>176</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>143</v>
+        <v>133</v>
       </c>
       <c r="G29" s="8" t="s">
-        <v>187</v>
+        <v>177</v>
       </c>
       <c r="H29" s="8" t="s">
-        <v>448</v>
+        <v>430</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="J29" s="8" t="s">
-        <v>189</v>
+        <v>179</v>
       </c>
       <c r="K29" s="8" t="s">
-        <v>190</v>
+        <v>180</v>
       </c>
       <c r="L29" s="8" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="M29" s="8" t="s">
-        <v>192</v>
+        <v>182</v>
       </c>
     </row>
     <row r="30" spans="1:13" ht="97" customHeight="1">
       <c r="A30" s="26" t="s">
-        <v>193</v>
+        <v>183</v>
       </c>
       <c r="B30" s="14" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C30" s="17"/>
       <c r="D30" s="17"/>
       <c r="E30" s="18" t="s">
-        <v>195</v>
+        <v>185</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>196</v>
+        <v>186</v>
       </c>
       <c r="G30" s="8" t="s">
-        <v>197</v>
+        <v>187</v>
       </c>
       <c r="H30" s="8" t="s">
-        <v>439</v>
+        <v>424</v>
       </c>
       <c r="I30" s="8" t="s">
-        <v>198</v>
+        <v>188</v>
       </c>
       <c r="J30" s="8" t="s">
+        <v>179</v>
+      </c>
+      <c r="K30" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="K30" s="8" t="s">
-        <v>199</v>
-      </c>
       <c r="L30" s="8" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="M30" s="8"/>
     </row>
@@ -3919,7 +3931,7 @@
       <c r="G31" s="28"/>
       <c r="H31" s="28"/>
       <c r="I31" s="28" t="s">
-        <v>201</v>
+        <v>191</v>
       </c>
       <c r="J31" s="28"/>
       <c r="K31" s="28"/>
@@ -3936,7 +3948,7 @@
       <c r="G32" s="28"/>
       <c r="H32" s="28"/>
       <c r="I32" s="28" t="s">
-        <v>202</v>
+        <v>192</v>
       </c>
       <c r="J32" s="28"/>
       <c r="K32" s="28"/>
@@ -4868,72 +4880,72 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.25" customHeight="1">
       <c r="A1" s="42" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="B1" s="42" t="s">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="C1" s="42" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D1" s="42" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="39" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>420</v>
+        <v>409</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>411</v>
+        <v>400</v>
       </c>
       <c r="E2" s="11"/>
     </row>
     <row r="3" spans="1:5" ht="26.25" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>209</v>
+        <v>199</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:5" ht="26.25" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>211</v>
+        <v>201</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>212</v>
+        <v>202</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>213</v>
+        <v>203</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="E4" s="11"/>
     </row>
     <row r="5" spans="1:5" ht="26.25" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>421</v>
+        <v>410</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>16</v>
@@ -4942,13 +4954,13 @@
     </row>
     <row r="6" spans="1:5" ht="15">
       <c r="A6" s="10" t="s">
-        <v>216</v>
+        <v>206</v>
       </c>
       <c r="B6" s="8" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
       <c r="C6" s="8" t="s">
-        <v>218</v>
+        <v>208</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>25</v>
@@ -4957,13 +4969,13 @@
     </row>
     <row r="7" spans="1:5" ht="15">
       <c r="A7" s="10" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="C7" s="8" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>32</v>
@@ -4972,106 +4984,106 @@
     </row>
     <row r="8" spans="1:5" ht="26.25" customHeight="1">
       <c r="A8" s="10" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>422</v>
+        <v>411</v>
       </c>
       <c r="C8" s="8" t="s">
-        <v>423</v>
+        <v>412</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="30">
       <c r="A9" s="10" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>424</v>
+        <v>413</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>425</v>
+        <v>414</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" customHeight="1">
       <c r="A10" s="10" t="s">
-        <v>224</v>
+        <v>214</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C10" s="8" t="s">
-        <v>226</v>
+        <v>216</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="E10" s="11"/>
     </row>
     <row r="11" spans="1:5" ht="26.25" customHeight="1">
       <c r="A11" s="10" t="s">
-        <v>227</v>
+        <v>217</v>
       </c>
       <c r="B11" s="8" t="s">
-        <v>228</v>
+        <v>218</v>
       </c>
       <c r="C11" s="8" t="s">
-        <v>229</v>
+        <v>219</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:5" ht="26.25" customHeight="1">
       <c r="A12" s="10" t="s">
-        <v>230</v>
+        <v>220</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>231</v>
+        <v>221</v>
       </c>
       <c r="C12" s="8" t="s">
-        <v>232</v>
+        <v>222</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E12" s="11"/>
     </row>
     <row r="13" spans="1:5" ht="15">
       <c r="A13" s="10" t="s">
-        <v>233</v>
+        <v>223</v>
       </c>
       <c r="B13" s="8" t="s">
-        <v>234</v>
+        <v>224</v>
       </c>
       <c r="C13" s="8" t="s">
-        <v>235</v>
+        <v>225</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E13" s="11"/>
     </row>
     <row r="14" spans="1:5" ht="38.25" customHeight="1">
       <c r="A14" s="10" t="s">
-        <v>236</v>
+        <v>226</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>237</v>
+        <v>227</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>238</v>
+        <v>228</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>410</v>
+        <v>399</v>
       </c>
       <c r="E14" s="11"/>
     </row>
@@ -5160,72 +5172,72 @@
   <sheetData>
     <row r="1" spans="1:4" ht="26.25" customHeight="1">
       <c r="A1" s="30" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="B1" s="30" t="s">
-        <v>239</v>
+        <v>229</v>
       </c>
       <c r="C1" s="30" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D1" s="30" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="39" customHeight="1">
       <c r="A2" s="10" t="s">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>241</v>
+        <v>231</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>242</v>
+        <v>232</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="39" customHeight="1">
       <c r="A3" s="10" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>245</v>
+        <v>235</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>246</v>
+        <v>236</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>247</v>
+        <v>237</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="39" customHeight="1">
       <c r="A4" s="10" t="s">
-        <v>248</v>
+        <v>238</v>
       </c>
       <c r="B4" s="8" t="s">
-        <v>249</v>
+        <v>239</v>
       </c>
       <c r="C4" s="8" t="s">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>251</v>
+        <v>241</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="26.25" customHeight="1">
       <c r="A5" s="10" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="B5" s="8" t="s">
-        <v>253</v>
+        <v>243</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>254</v>
+        <v>244</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>255</v>
+        <v>245</v>
       </c>
     </row>
   </sheetData>
@@ -5247,150 +5259,150 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.25" customHeight="1">
       <c r="A1" s="31" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>256</v>
+        <v>246</v>
       </c>
       <c r="C1" s="31" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D1" s="31" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="65.25" customHeight="1">
       <c r="A2" s="12" t="s">
-        <v>257</v>
+        <v>247</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>427</v>
+        <v>416</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>258</v>
+        <v>248</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>259</v>
+        <v>249</v>
       </c>
       <c r="E2" s="11"/>
     </row>
     <row r="3" spans="1:5" ht="26.25" customHeight="1">
       <c r="A3" s="12" t="s">
-        <v>260</v>
+        <v>250</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>261</v>
+        <v>251</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>262</v>
+        <v>252</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>263</v>
+        <v>253</v>
       </c>
       <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:5" ht="26.25" customHeight="1">
       <c r="A4" s="12" t="s">
-        <v>264</v>
+        <v>254</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>265</v>
+        <v>255</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>266</v>
+        <v>256</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E4" s="11"/>
     </row>
     <row r="5" spans="1:5" ht="26.25" customHeight="1">
       <c r="A5" s="12" t="s">
-        <v>267</v>
+        <v>257</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>268</v>
+        <v>258</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>269</v>
+        <v>259</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="E5" s="11"/>
     </row>
     <row r="6" spans="1:5" ht="30">
       <c r="A6" s="12" t="s">
-        <v>270</v>
+        <v>260</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>414</v>
+        <v>403</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>413</v>
+        <v>402</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="15">
       <c r="A7" s="12" t="s">
-        <v>271</v>
+        <v>261</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>272</v>
+        <v>262</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>273</v>
+        <v>263</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="15">
       <c r="A8" s="12" t="s">
-        <v>274</v>
+        <v>264</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>275</v>
+        <v>265</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>276</v>
+        <v>266</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="26.25" customHeight="1">
       <c r="A9" s="12" t="s">
-        <v>277</v>
+        <v>267</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>278</v>
+        <v>268</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>279</v>
+        <v>269</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="15">
       <c r="A10" s="12" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>282</v>
+        <v>272</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="E10" s="11"/>
     </row>
@@ -5413,150 +5425,150 @@
   <sheetData>
     <row r="1" spans="1:5" ht="26.25" customHeight="1">
       <c r="A1" s="31" t="s">
-        <v>203</v>
+        <v>193</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>283</v>
+        <v>273</v>
       </c>
       <c r="C1" s="31" t="s">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="D1" s="31" t="s">
-        <v>206</v>
+        <v>196</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="26.25" customHeight="1">
       <c r="A2" s="13" t="s">
-        <v>284</v>
+        <v>274</v>
       </c>
       <c r="B2" s="9" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="C2" s="9" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="D2" s="12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E2" s="11"/>
     </row>
     <row r="3" spans="1:5" ht="15">
       <c r="A3" s="13" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>289</v>
+        <v>279</v>
       </c>
       <c r="D3" s="12" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E3" s="11"/>
     </row>
     <row r="4" spans="1:5" ht="15">
       <c r="A4" s="13" t="s">
-        <v>290</v>
+        <v>280</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>291</v>
+        <v>281</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>292</v>
+        <v>282</v>
       </c>
       <c r="D4" s="12" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="E4" s="11"/>
     </row>
     <row r="5" spans="1:5" ht="15">
       <c r="A5" s="13" t="s">
-        <v>293</v>
+        <v>283</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>294</v>
+        <v>284</v>
       </c>
       <c r="C5" s="9" t="s">
-        <v>295</v>
+        <v>285</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E5" s="11"/>
     </row>
     <row r="6" spans="1:5" ht="26.25" customHeight="1">
       <c r="A6" s="13" t="s">
-        <v>296</v>
+        <v>286</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>297</v>
+        <v>287</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>298</v>
+        <v>288</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>299</v>
+        <v>289</v>
       </c>
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="26.25" customHeight="1">
       <c r="A7" s="13" t="s">
-        <v>300</v>
+        <v>290</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>301</v>
+        <v>291</v>
       </c>
       <c r="C7" s="9" t="s">
-        <v>302</v>
+        <v>292</v>
       </c>
       <c r="D7" s="12" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="15">
       <c r="A8" s="13" t="s">
-        <v>303</v>
+        <v>293</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>304</v>
+        <v>294</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>305</v>
+        <v>295</v>
       </c>
       <c r="D8" s="12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="26.25" customHeight="1">
       <c r="A9" s="13" t="s">
-        <v>306</v>
+        <v>296</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>307</v>
+        <v>297</v>
       </c>
       <c r="C9" s="9" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" customHeight="1">
       <c r="A10" s="13" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>310</v>
+        <v>300</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>308</v>
+        <v>298</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="E10" s="11"/>
     </row>
@@ -5599,26 +5611,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28" customHeight="1">
-      <c r="A1" s="49" t="s">
-        <v>311</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
+      <c r="A1" s="50" t="s">
+        <v>301</v>
+      </c>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1">
-      <c r="A2" s="53" t="s">
-        <v>312</v>
-      </c>
-      <c r="B2" s="48"/>
-      <c r="C2" s="48"/>
-      <c r="D2" s="48"/>
-      <c r="E2" s="48"/>
-      <c r="F2" s="48"/>
-      <c r="G2" s="48"/>
+      <c r="A2" s="54" t="s">
+        <v>302</v>
+      </c>
+      <c r="B2" s="49"/>
+      <c r="C2" s="49"/>
+      <c r="D2" s="49"/>
+      <c r="E2" s="49"/>
+      <c r="F2" s="49"/>
+      <c r="G2" s="49"/>
     </row>
     <row r="3" spans="1:7" ht="8.25" customHeight="1"/>
     <row r="4" spans="1:7" ht="28" customHeight="1">
@@ -5626,34 +5638,34 @@
         <v>4</v>
       </c>
       <c r="B4" s="21" t="s">
-        <v>313</v>
+        <v>303</v>
       </c>
       <c r="C4" s="21" t="s">
-        <v>314</v>
+        <v>304</v>
       </c>
       <c r="D4" s="21" t="s">
-        <v>315</v>
+        <v>305</v>
       </c>
       <c r="E4" s="21" t="s">
-        <v>316</v>
+        <v>306</v>
       </c>
       <c r="F4" s="21" t="s">
-        <v>317</v>
+        <v>307</v>
       </c>
       <c r="G4" s="21" t="s">
-        <v>318</v>
+        <v>308</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A5" s="50" t="s">
-        <v>319</v>
-      </c>
-      <c r="B5" s="51"/>
-      <c r="C5" s="51"/>
-      <c r="D5" s="51"/>
-      <c r="E5" s="51"/>
-      <c r="F5" s="51"/>
-      <c r="G5" s="52"/>
+      <c r="A5" s="51" t="s">
+        <v>309</v>
+      </c>
+      <c r="B5" s="52"/>
+      <c r="C5" s="52"/>
+      <c r="D5" s="52"/>
+      <c r="E5" s="52"/>
+      <c r="F5" s="52"/>
+      <c r="G5" s="53"/>
     </row>
     <row r="6" spans="1:7" ht="75" customHeight="1">
       <c r="A6" s="43">
@@ -5663,19 +5675,19 @@
         <v>17</v>
       </c>
       <c r="C6" s="44" t="s">
-        <v>320</v>
+        <v>310</v>
       </c>
       <c r="D6" s="44" t="s">
-        <v>321</v>
+        <v>311</v>
       </c>
       <c r="E6" s="44" t="s">
-        <v>322</v>
+        <v>312</v>
       </c>
       <c r="F6" s="44" t="s">
-        <v>323</v>
+        <v>313</v>
       </c>
       <c r="G6" s="44" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="75" customHeight="1">
@@ -5686,19 +5698,19 @@
         <v>26</v>
       </c>
       <c r="C7" s="46" t="s">
-        <v>325</v>
+        <v>315</v>
       </c>
       <c r="D7" s="46" t="s">
-        <v>326</v>
+        <v>316</v>
       </c>
       <c r="E7" s="46" t="s">
-        <v>327</v>
+        <v>317</v>
       </c>
       <c r="F7" s="46" t="s">
-        <v>328</v>
+        <v>318</v>
       </c>
       <c r="G7" s="46" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="8" spans="1:7" ht="75" customHeight="1">
@@ -5709,19 +5721,19 @@
         <v>33</v>
       </c>
       <c r="C8" s="44" t="s">
-        <v>329</v>
+        <v>319</v>
       </c>
       <c r="D8" s="44" t="s">
-        <v>330</v>
+        <v>320</v>
       </c>
       <c r="E8" s="44" t="s">
-        <v>331</v>
+        <v>321</v>
       </c>
       <c r="F8" s="44" t="s">
-        <v>332</v>
+        <v>322</v>
       </c>
       <c r="G8" s="44" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="9" spans="1:7" ht="75" customHeight="1">
@@ -5732,19 +5744,19 @@
         <v>41</v>
       </c>
       <c r="C9" s="46" t="s">
-        <v>333</v>
+        <v>323</v>
       </c>
       <c r="D9" s="46" t="s">
-        <v>426</v>
+        <v>415</v>
       </c>
       <c r="E9" s="46" t="s">
-        <v>334</v>
+        <v>324</v>
       </c>
       <c r="F9" s="46" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="G9" s="46" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
     </row>
     <row r="10" spans="1:7" ht="75" customHeight="1">
@@ -5752,22 +5764,22 @@
         <v>5</v>
       </c>
       <c r="B10" s="43" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C10" s="44" t="s">
-        <v>337</v>
+        <v>327</v>
       </c>
       <c r="D10" s="44" t="s">
-        <v>338</v>
+        <v>328</v>
       </c>
       <c r="E10" s="44" t="s">
-        <v>339</v>
+        <v>329</v>
       </c>
       <c r="F10" s="44" t="s">
-        <v>340</v>
+        <v>330</v>
       </c>
       <c r="G10" s="44" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
     <row r="11" spans="1:7" ht="75" customHeight="1">
@@ -5775,56 +5787,56 @@
         <v>6</v>
       </c>
       <c r="B11" s="45" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="46" t="s">
-        <v>342</v>
+        <v>332</v>
       </c>
       <c r="D11" s="46" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="E11" s="46" t="s">
-        <v>344</v>
+        <v>334</v>
       </c>
       <c r="F11" s="46" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="G11" s="46" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="12" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A12" s="50" t="s">
-        <v>346</v>
-      </c>
-      <c r="B12" s="51"/>
-      <c r="C12" s="51"/>
-      <c r="D12" s="51"/>
-      <c r="E12" s="51"/>
-      <c r="F12" s="51"/>
-      <c r="G12" s="52"/>
+      <c r="A12" s="51" t="s">
+        <v>336</v>
+      </c>
+      <c r="B12" s="52"/>
+      <c r="C12" s="52"/>
+      <c r="D12" s="52"/>
+      <c r="E12" s="52"/>
+      <c r="F12" s="52"/>
+      <c r="G12" s="53"/>
     </row>
     <row r="13" spans="1:7" ht="75" customHeight="1">
       <c r="A13" s="24">
         <v>7</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C13" s="25" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D13" s="25" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="E13" s="25" t="s">
-        <v>348</v>
+        <v>338</v>
       </c>
       <c r="F13" s="25" t="s">
-        <v>349</v>
+        <v>339</v>
       </c>
       <c r="G13" s="25" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
     </row>
     <row r="14" spans="1:7" ht="75" customHeight="1">
@@ -5832,22 +5844,22 @@
         <v>8</v>
       </c>
       <c r="B14" s="22" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C14" s="23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="D14" s="23" t="s">
-        <v>350</v>
+        <v>340</v>
       </c>
       <c r="E14" s="23" t="s">
-        <v>351</v>
+        <v>341</v>
       </c>
       <c r="F14" s="23" t="s">
-        <v>352</v>
+        <v>342</v>
       </c>
       <c r="G14" s="23" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="75" customHeight="1">
@@ -5855,22 +5867,22 @@
         <v>9</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C15" s="25" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="D15" s="25" t="s">
-        <v>353</v>
+        <v>343</v>
       </c>
       <c r="E15" s="25" t="s">
-        <v>354</v>
+        <v>344</v>
       </c>
       <c r="F15" s="25" t="s">
-        <v>355</v>
+        <v>345</v>
       </c>
       <c r="G15" s="25" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="16" spans="1:7" ht="75" customHeight="1">
@@ -5878,22 +5890,22 @@
         <v>10</v>
       </c>
       <c r="B16" s="22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C16" s="23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="D16" s="23" t="s">
-        <v>356</v>
+        <v>346</v>
       </c>
       <c r="E16" s="23" t="s">
-        <v>357</v>
+        <v>347</v>
       </c>
       <c r="F16" s="23" t="s">
-        <v>358</v>
+        <v>348</v>
       </c>
       <c r="G16" s="23" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="75" customHeight="1">
@@ -5901,22 +5913,22 @@
         <v>11</v>
       </c>
       <c r="B17" s="24" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C17" s="25" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D17" s="25" t="s">
-        <v>359</v>
+        <v>349</v>
       </c>
       <c r="E17" s="25" t="s">
-        <v>360</v>
+        <v>350</v>
       </c>
       <c r="F17" s="25" t="s">
-        <v>361</v>
+        <v>351</v>
       </c>
       <c r="G17" s="25" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="75" customHeight="1">
@@ -5924,22 +5936,22 @@
         <v>12</v>
       </c>
       <c r="B18" s="22" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C18" s="23" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D18" s="23" t="s">
-        <v>362</v>
+        <v>352</v>
       </c>
       <c r="E18" s="23" t="s">
-        <v>363</v>
+        <v>353</v>
       </c>
       <c r="F18" s="23" t="s">
-        <v>364</v>
+        <v>354</v>
       </c>
       <c r="G18" s="23" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="19" spans="1:7" ht="75" customHeight="1">
@@ -5947,22 +5959,22 @@
         <v>13</v>
       </c>
       <c r="B19" s="24" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>365</v>
+        <v>355</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="75" customHeight="1">
@@ -5970,56 +5982,56 @@
         <v>14</v>
       </c>
       <c r="B20" s="22" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="C20" s="23" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="D20" s="23" t="s">
-        <v>370</v>
+        <v>360</v>
       </c>
       <c r="E20" s="23" t="s">
-        <v>371</v>
+        <v>361</v>
       </c>
       <c r="F20" s="23" t="s">
-        <v>372</v>
+        <v>362</v>
       </c>
       <c r="G20" s="23" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A21" s="50" t="s">
-        <v>373</v>
-      </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
-      <c r="G21" s="52"/>
+      <c r="A21" s="51" t="s">
+        <v>363</v>
+      </c>
+      <c r="B21" s="52"/>
+      <c r="C21" s="52"/>
+      <c r="D21" s="52"/>
+      <c r="E21" s="52"/>
+      <c r="F21" s="52"/>
+      <c r="G21" s="53"/>
     </row>
     <row r="22" spans="1:7" ht="75" customHeight="1">
       <c r="A22" s="22">
         <v>15</v>
       </c>
       <c r="B22" s="22" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C22" s="23" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="D22" s="23" t="s">
-        <v>374</v>
+        <v>364</v>
       </c>
       <c r="E22" s="23" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="F22" s="23" t="s">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="G22" s="23" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="23" spans="1:7" ht="75" customHeight="1">
@@ -6027,56 +6039,56 @@
         <v>16</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>124</v>
+        <v>114</v>
       </c>
       <c r="C23" s="25" t="s">
-        <v>125</v>
+        <v>115</v>
       </c>
       <c r="D23" s="25" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>378</v>
+        <v>368</v>
       </c>
       <c r="F23" s="25" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="G23" s="25" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="20.25" customHeight="1">
-      <c r="A24" s="50" t="s">
-        <v>380</v>
-      </c>
-      <c r="B24" s="51"/>
-      <c r="C24" s="51"/>
-      <c r="D24" s="51"/>
-      <c r="E24" s="51"/>
-      <c r="F24" s="51"/>
-      <c r="G24" s="52"/>
+      <c r="A24" s="51" t="s">
+        <v>370</v>
+      </c>
+      <c r="B24" s="52"/>
+      <c r="C24" s="52"/>
+      <c r="D24" s="52"/>
+      <c r="E24" s="52"/>
+      <c r="F24" s="52"/>
+      <c r="G24" s="53"/>
     </row>
     <row r="25" spans="1:7" ht="75" customHeight="1">
       <c r="A25" s="24">
         <v>17</v>
       </c>
       <c r="B25" s="24" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="C25" s="25" t="s">
-        <v>381</v>
+        <v>371</v>
       </c>
       <c r="D25" s="25" t="s">
-        <v>382</v>
+        <v>372</v>
       </c>
       <c r="E25" s="25" t="s">
-        <v>383</v>
+        <v>373</v>
       </c>
       <c r="F25" s="25" t="s">
-        <v>384</v>
+        <v>374</v>
       </c>
       <c r="G25" s="25" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
     </row>
     <row r="26" spans="1:7" ht="75" customHeight="1">
@@ -6084,22 +6096,22 @@
         <v>18</v>
       </c>
       <c r="B26" s="22" t="s">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C26" s="23" t="s">
-        <v>385</v>
+        <v>375</v>
       </c>
       <c r="D26" s="23" t="s">
-        <v>386</v>
+        <v>376</v>
       </c>
       <c r="E26" s="23" t="s">
-        <v>387</v>
+        <v>377</v>
       </c>
       <c r="F26" s="23" t="s">
-        <v>335</v>
+        <v>325</v>
       </c>
       <c r="G26" s="23" t="s">
-        <v>336</v>
+        <v>326</v>
       </c>
     </row>
     <row r="27" spans="1:7" ht="75" customHeight="1">
@@ -6107,22 +6119,22 @@
         <v>19</v>
       </c>
       <c r="B27" s="24" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
       <c r="C27" s="25" t="s">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="D27" s="25" t="s">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="E27" s="25" t="s">
-        <v>389</v>
+        <v>379</v>
       </c>
       <c r="F27" s="25" t="s">
-        <v>244</v>
+        <v>234</v>
       </c>
       <c r="G27" s="25" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="75" customHeight="1">
@@ -6130,22 +6142,22 @@
         <v>20</v>
       </c>
       <c r="B28" s="22" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C28" s="23" t="s">
-        <v>390</v>
+        <v>380</v>
       </c>
       <c r="D28" s="23" t="s">
-        <v>391</v>
+        <v>381</v>
       </c>
       <c r="E28" s="23" t="s">
-        <v>392</v>
+        <v>382</v>
       </c>
       <c r="F28" s="23" t="s">
-        <v>393</v>
+        <v>383</v>
       </c>
       <c r="G28" s="23" t="s">
-        <v>324</v>
+        <v>314</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="75" customHeight="1">
@@ -6153,22 +6165,22 @@
         <v>21</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>167</v>
+        <v>157</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>394</v>
+        <v>384</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>395</v>
+        <v>385</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="F29" s="25" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="G29" s="25" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="75" customHeight="1">
@@ -6176,22 +6188,22 @@
         <v>22</v>
       </c>
       <c r="B30" s="22" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="C30" s="23" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="D30" s="23" t="s">
-        <v>398</v>
+        <v>388</v>
       </c>
       <c r="E30" s="23" t="s">
-        <v>399</v>
+        <v>389</v>
       </c>
       <c r="F30" s="23" t="s">
-        <v>252</v>
+        <v>242</v>
       </c>
       <c r="G30" s="23" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="75" customHeight="1">
@@ -6199,22 +6211,22 @@
         <v>23</v>
       </c>
       <c r="B31" s="24" t="s">
-        <v>184</v>
+        <v>174</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>400</v>
+        <v>390</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>401</v>
+        <v>391</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>402</v>
+        <v>392</v>
       </c>
       <c r="F31" s="25" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="G31" s="25" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="75" customHeight="1">
@@ -6222,22 +6234,22 @@
         <v>24</v>
       </c>
       <c r="B32" s="22" t="s">
-        <v>194</v>
+        <v>184</v>
       </c>
       <c r="C32" s="23" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="D32" s="23" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="E32" s="23" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="F32" s="23" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="G32" s="23" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -6265,6 +6277,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c58ecc89-2e47-4dee-a93d-93f030b574a9" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b65048e3-dffa-4253-8538-8fa05818bc09">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="ドキュメント" ma:contentTypeID="0x01010060506946A466D34388C42452DB951185" ma:contentTypeVersion="12" ma:contentTypeDescription="新しいドキュメントを作成します。" ma:contentTypeScope="" ma:versionID="e7f9e42ee651ece8a11972bb003729bf">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b65048e3-dffa-4253-8538-8fa05818bc09" xmlns:ns3="c58ecc89-2e47-4dee-a93d-93f030b574a9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d8836cf6f3c39efd57cd52c4c2225720" ns2:_="" ns3:_="">
     <xsd:import namespace="b65048e3-dffa-4253-8538-8fa05818bc09"/>
@@ -6465,17 +6488,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c58ecc89-2e47-4dee-a93d-93f030b574a9" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b65048e3-dffa-4253-8538-8fa05818bc09">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{970AD663-EFBF-4F4F-BFD6-44D1A5F56D8A}">
   <ds:schemaRefs>
@@ -6485,6 +6497,23 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB9B0F14-3F24-4310-9574-73C25A41EBCC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="c58ecc89-2e47-4dee-a93d-93f030b574a9"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="b65048e3-dffa-4253-8538-8fa05818bc09"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B81A579-D803-4880-9E6F-9314008CBC69}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -6501,21 +6530,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EB9B0F14-3F24-4310-9574-73C25A41EBCC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="c58ecc89-2e47-4dee-a93d-93f030b574a9"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="b65048e3-dffa-4253-8538-8fa05818bc09"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>